<commit_message>
chore(data): run hebdo 2026-04-30
</commit_message>
<xml_diff>
--- a/exports/education/etablissements_education_france.xlsx
+++ b/exports/education/etablissements_education_france.xlsx
@@ -740,7 +740,7 @@
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-04-24 15:01:44</t>
+          <t>2026-04-30 12:29:46</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
       </c>
       <c r="P3" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24 15:01:46</t>
+          <t>2026-04-30 12:29:51</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>2026-04-24 15:01:50</t>
+          <t>2026-04-30 12:29:53</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24 15:01:55</t>
+          <t>2026-04-30 12:29:58</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>2026-04-24 15:01:58</t>
+          <t>2026-04-30 12:30:02</t>
         </is>
       </c>
     </row>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24 15:02:03</t>
+          <t>2026-04-30 12:30:05</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>2026-04-24 15:02:10</t>
+          <t>2026-04-30 12:30:09</t>
         </is>
       </c>
     </row>
@@ -1290,7 +1290,7 @@
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24 15:02:15</t>
+          <t>2026-04-30 12:30:11</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>2026-04-24 15:02:18</t>
+          <t>2026-04-30 12:30:16</t>
         </is>
       </c>
     </row>
@@ -1450,7 +1450,7 @@
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24 15:02:22</t>
+          <t>2026-04-30 12:30:18</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>2026-04-24 15:02:27</t>
+          <t>2026-04-30 12:30:21</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24 15:02:30</t>
+          <t>2026-04-30 12:30:25</t>
         </is>
       </c>
     </row>

</xml_diff>